<commit_message>
Updated AP CS tab
</commit_message>
<xml_diff>
--- a/data/cs_degree_trends.xlsx
+++ b/data/cs_degree_trends.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoregon-my.sharepoint.com/personal/mcui_uoregon_edu/Documents/UO_QRME Program/QRME PhD program/Winter_26_EDLD 640/Student_Access_to_AP_CS/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D66052-42A5-FF44-AA46-AA13BFE89726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{64D66052-42A5-FF44-AA46-AA13BFE89726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88E43D73-990F-C440-ADCC-552CF63AE938}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="25600" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,9 +68,6 @@
     <t>NOTE: Data in this table represent the 50 states and the District of Columbia. Data are for degree-granting institutions and U.S. service academies. Degree-granting institutions grant associate’s or higher degrees and participate in Title IV federal financial aid programs. Data in this table are based on the 2020 Classification of Instructional Programs. Some data have been revised from previously published figures.</t>
   </si>
   <si>
-    <t>SOURCE: U.S. Department of Education, National Center for Education Statistics, Earned Degrees Conferred, 1964-65 through 1969-70; Higher Education General Information Survey (HEGIS), "Degrees and Other Formal Awards Conferred" surveys, 1970-71 through 1985-86; Integrated Postsecondary Education Data System (IPEDS), "Completions Survey" (IPEDS-C:87-99); Completions component, IPEDS Fall 2000 through Fall 2021 (final data) and Fall 2022 (provisional data).  (This table was prepared November 2023.)</t>
-  </si>
-  <si>
     <t>Table 325.35. Degrees in computer and information sciences conferred by postsecondary institutions, by level of degree and sex of 
               student: Academic years 1964-65 through 2021-22</t>
   </si>
@@ -265,6 +262,9 @@
   </si>
   <si>
     <t>  2016-17 to 2021-22</t>
+  </si>
+  <si>
+    <t>SOURCE: U.S. Department of Education, National Center for Education Statistics, Earned Degrees Conferred, 1964-65 through 1969-70; Higher Education General Information SurveDegry (HEGIS), "Degrees and Other Formal Awards Conferred" surveys, 1970-71 through 1985-86; Integrated Postsecondary Education Data System (IPEDS), "Completions Survey" (IPEDS-C:87-99); Completions component, IPEDS Fall 2000 through Fall 2021 (final data) and Fall 2022 (provisional data).  (This table was prepared November 2023.)</t>
   </si>
 </sst>
 </file>
@@ -391,6 +391,9 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -404,9 +407,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -726,132 +726,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+    </row>
+    <row r="2" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="L2" s="14" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="I3" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="J3" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="K3" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="L3" s="14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-    </row>
-    <row r="2" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="20" t="s">
-        <v>6</v>
-      </c>
-      <c r="I2" s="20" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="L2" s="20" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="19" t="s">
+      <c r="C4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="H4" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="J4" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="K4" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="20" t="s">
-        <v>2</v>
-      </c>
-      <c r="H3" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="I3" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="J3" s="20" t="s">
-        <v>2</v>
-      </c>
-      <c r="K3" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="L3" s="20" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="F4" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="20" t="s">
-        <v>2</v>
-      </c>
-      <c r="H4" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="J4" s="20" t="s">
-        <v>2</v>
-      </c>
-      <c r="K4" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="L4" s="20" t="s">
+      <c r="L4" s="14" t="s">
         <v>4</v>
       </c>
     </row>
@@ -895,13 +895,13 @@
     </row>
     <row r="6" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" s="5">
         <v>87</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D6" s="5">
         <v>83</v>
@@ -933,7 +933,7 @@
     </row>
     <row r="7" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="5">
         <v>89</v>
@@ -971,7 +971,7 @@
     </row>
     <row r="8" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="5">
         <v>222</v>
@@ -1009,7 +1009,7 @@
     </row>
     <row r="9" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="5">
         <v>459</v>
@@ -1047,7 +1047,7 @@
     </row>
     <row r="10" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="5">
         <v>933</v>
@@ -1085,7 +1085,7 @@
     </row>
     <row r="11" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" s="5">
         <v>1544</v>
@@ -1123,7 +1123,7 @@
     </row>
     <row r="12" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="5">
         <v>2388</v>
@@ -1161,7 +1161,7 @@
     </row>
     <row r="13" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="5">
         <v>3402</v>
@@ -1199,7 +1199,7 @@
     </row>
     <row r="14" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="5">
         <v>4304</v>
@@ -1237,7 +1237,7 @@
     </row>
     <row r="15" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" s="5">
         <v>4756</v>
@@ -1275,7 +1275,7 @@
     </row>
     <row r="16" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B16" s="5">
         <v>5033</v>
@@ -1313,7 +1313,7 @@
     </row>
     <row r="17" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B17" s="5">
         <v>5652</v>
@@ -1351,7 +1351,7 @@
     </row>
     <row r="18" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B18" s="5">
         <v>6407</v>
@@ -1389,7 +1389,7 @@
     </row>
     <row r="19" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B19" s="5">
         <v>7201</v>
@@ -1427,7 +1427,7 @@
     </row>
     <row r="20" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B20" s="5">
         <v>8719</v>
@@ -1465,7 +1465,7 @@
     </row>
     <row r="21" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B21" s="5">
         <v>11154</v>
@@ -1503,7 +1503,7 @@
     </row>
     <row r="22" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B22" s="5">
         <v>15121</v>
@@ -1541,7 +1541,7 @@
     </row>
     <row r="23" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B23" s="5">
         <v>20267</v>
@@ -1579,7 +1579,7 @@
     </row>
     <row r="24" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24" s="5">
         <v>24565</v>
@@ -1617,7 +1617,7 @@
     </row>
     <row r="25" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B25" s="5">
         <v>32439</v>
@@ -1655,7 +1655,7 @@
     </row>
     <row r="26" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B26" s="5">
         <v>39121</v>
@@ -1693,7 +1693,7 @@
     </row>
     <row r="27" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B27" s="5">
         <v>42337</v>
@@ -1731,7 +1731,7 @@
     </row>
     <row r="28" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B28" s="5">
         <v>39767</v>
@@ -1769,7 +1769,7 @@
     </row>
     <row r="29" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B29" s="5">
         <v>34651</v>
@@ -1807,7 +1807,7 @@
     </row>
     <row r="30" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B30" s="5">
         <v>30560</v>
@@ -1845,7 +1845,7 @@
     </row>
     <row r="31" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B31" s="5">
         <v>27347</v>
@@ -1883,7 +1883,7 @@
     </row>
     <row r="32" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B32" s="5">
         <v>25159</v>
@@ -1921,7 +1921,7 @@
     </row>
     <row r="33" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B33" s="5">
         <v>24821</v>
@@ -1959,7 +1959,7 @@
     </row>
     <row r="34" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B34" s="5">
         <v>24519</v>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="35" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B35" s="5">
         <v>24527</v>
@@ -2035,7 +2035,7 @@
     </row>
     <row r="36" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B36" s="5">
         <v>24737</v>
@@ -2073,7 +2073,7 @@
     </row>
     <row r="37" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B37" s="5">
         <v>24506</v>
@@ -2111,7 +2111,7 @@
     </row>
     <row r="38" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B38" s="5">
         <v>25422</v>
@@ -2149,7 +2149,7 @@
     </row>
     <row r="39" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B39" s="5">
         <v>27829</v>
@@ -2187,7 +2187,7 @@
     </row>
     <row r="40" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B40" s="5">
         <v>30552</v>
@@ -2225,7 +2225,7 @@
     </row>
     <row r="41" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B41" s="5">
         <v>37788</v>
@@ -2263,7 +2263,7 @@
     </row>
     <row r="42" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B42" s="5">
         <v>44142</v>
@@ -2301,7 +2301,7 @@
     </row>
     <row r="43" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B43" s="5">
         <v>50365</v>
@@ -2339,7 +2339,7 @@
     </row>
     <row r="44" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B44" s="5">
         <v>57433</v>
@@ -2377,7 +2377,7 @@
     </row>
     <row r="45" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B45" s="5">
         <v>59488</v>
@@ -2415,7 +2415,7 @@
     </row>
     <row r="46" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B46" s="5">
         <v>54111</v>
@@ -2453,7 +2453,7 @@
     </row>
     <row r="47" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B47" s="5">
         <v>47702</v>
@@ -2491,7 +2491,7 @@
     </row>
     <row r="48" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B48" s="5">
         <v>42164</v>
@@ -2529,7 +2529,7 @@
     </row>
     <row r="49" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B49" s="5">
         <v>38523</v>
@@ -2567,7 +2567,7 @@
     </row>
     <row r="50" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B50" s="5">
         <v>37992</v>
@@ -2605,7 +2605,7 @@
     </row>
     <row r="51" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B51" s="5">
         <v>39593</v>
@@ -2643,7 +2643,7 @@
     </row>
     <row r="52" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B52" s="5">
         <v>43066</v>
@@ -2681,7 +2681,7 @@
     </row>
     <row r="53" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B53" s="5">
         <v>47406</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="54" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B54" s="5">
         <v>50961</v>
@@ -2757,7 +2757,7 @@
     </row>
     <row r="55" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B55" s="5">
         <v>55271</v>
@@ -2795,7 +2795,7 @@
     </row>
     <row r="56" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B56" s="5">
         <v>59586</v>
@@ -2833,7 +2833,7 @@
     </row>
     <row r="57" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B57" s="5">
         <v>64402</v>
@@ -2871,7 +2871,7 @@
     </row>
     <row r="58" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B58" s="5">
         <v>71416</v>
@@ -2909,7 +2909,7 @@
     </row>
     <row r="59" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B59" s="5">
         <v>79597</v>
@@ -2947,7 +2947,7 @@
     </row>
     <row r="60" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B60" s="5">
         <v>88638</v>
@@ -2985,7 +2985,7 @@
     </row>
     <row r="61" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B61" s="5">
         <v>97054</v>
@@ -3023,7 +3023,7 @@
     </row>
     <row r="62" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B62" s="5">
         <v>104883</v>
@@ -3061,7 +3061,7 @@
     </row>
     <row r="63" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B63" s="9">
         <v>108503</v>
@@ -3099,7 +3099,7 @@
     </row>
     <row r="64" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="6"/>
@@ -3115,13 +3115,13 @@
     </row>
     <row r="65" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B65" s="7">
         <v>50.647597350546349</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D65" s="7">
         <v>48.889060727910092</v>
@@ -3130,7 +3130,7 @@
         <v>58.571428571428577</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G65" s="7">
         <v>122.4755077658303</v>
@@ -3153,13 +3153,13 @@
     </row>
     <row r="66" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B66" s="12">
         <v>51.930939845412787</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D66" s="12">
         <v>45.354292540207403</v>
@@ -3168,7 +3168,7 @@
         <v>79.755365121218773</v>
       </c>
       <c r="F66" s="13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G66" s="12">
         <v>10.27860717891436</v>
@@ -3190,76 +3190,71 @@
       </c>
     </row>
     <row r="67" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="14" t="s">
+      <c r="A67" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B67" s="15"/>
-      <c r="C67" s="15"/>
-      <c r="D67" s="15"/>
-      <c r="E67" s="15"/>
-      <c r="F67" s="15"/>
-      <c r="G67" s="15"/>
-      <c r="H67" s="15"/>
-      <c r="I67" s="15"/>
-      <c r="J67" s="15"/>
-      <c r="K67" s="15"/>
-      <c r="L67" s="15"/>
+      <c r="B67" s="16"/>
+      <c r="C67" s="16"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+      <c r="G67" s="16"/>
+      <c r="H67" s="16"/>
+      <c r="I67" s="16"/>
+      <c r="J67" s="16"/>
+      <c r="K67" s="16"/>
+      <c r="L67" s="16"/>
     </row>
     <row r="68" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="14" t="s">
+      <c r="A68" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B68" s="15"/>
-      <c r="C68" s="15"/>
-      <c r="D68" s="15"/>
-      <c r="E68" s="15"/>
-      <c r="F68" s="15"/>
-      <c r="G68" s="15"/>
-      <c r="H68" s="15"/>
-      <c r="I68" s="15"/>
-      <c r="J68" s="15"/>
-      <c r="K68" s="15"/>
-      <c r="L68" s="15"/>
+      <c r="B68" s="16"/>
+      <c r="C68" s="16"/>
+      <c r="D68" s="16"/>
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+      <c r="G68" s="16"/>
+      <c r="H68" s="16"/>
+      <c r="I68" s="16"/>
+      <c r="J68" s="16"/>
+      <c r="K68" s="16"/>
+      <c r="L68" s="16"/>
     </row>
     <row r="69" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="14" t="s">
+      <c r="A69" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B69" s="15"/>
-      <c r="C69" s="15"/>
-      <c r="D69" s="15"/>
-      <c r="E69" s="15"/>
-      <c r="F69" s="15"/>
-      <c r="G69" s="15"/>
-      <c r="H69" s="15"/>
-      <c r="I69" s="15"/>
-      <c r="J69" s="15"/>
-      <c r="K69" s="15"/>
-      <c r="L69" s="15"/>
+      <c r="B69" s="16"/>
+      <c r="C69" s="16"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
+      <c r="G69" s="16"/>
+      <c r="H69" s="16"/>
+      <c r="I69" s="16"/>
+      <c r="J69" s="16"/>
+      <c r="K69" s="16"/>
+      <c r="L69" s="16"/>
     </row>
     <row r="70" spans="1:12" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B70" s="15"/>
-      <c r="C70" s="15"/>
-      <c r="D70" s="15"/>
-      <c r="E70" s="15"/>
-      <c r="F70" s="15"/>
-      <c r="G70" s="15"/>
-      <c r="H70" s="15"/>
-      <c r="I70" s="15"/>
-      <c r="J70" s="15"/>
-      <c r="K70" s="15"/>
-      <c r="L70" s="15"/>
+      <c r="A70" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="B70" s="16"/>
+      <c r="C70" s="16"/>
+      <c r="D70" s="16"/>
+      <c r="E70" s="16"/>
+      <c r="F70" s="16"/>
+      <c r="G70" s="16"/>
+      <c r="H70" s="16"/>
+      <c r="I70" s="16"/>
+      <c r="J70" s="16"/>
+      <c r="K70" s="16"/>
+      <c r="L70" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="A67:L67"/>
-    <mergeCell ref="A68:L68"/>
-    <mergeCell ref="A69:L69"/>
-    <mergeCell ref="A70:L70"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:F2"/>
@@ -3274,6 +3269,11 @@
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="J3:J4"/>
     <mergeCell ref="K3:K4"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="A67:L67"/>
+    <mergeCell ref="A68:L68"/>
+    <mergeCell ref="A69:L69"/>
+    <mergeCell ref="A70:L70"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>